<commit_message>
Implement email notification with Excel report attachment
</commit_message>
<xml_diff>
--- a/src/main/resources/priceReport.xlsx
+++ b/src/main/resources/priceReport.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="20">
   <si>
     <t>Product Name</t>
   </si>
@@ -51,9 +51,6 @@
   </si>
   <si>
     <t>Anarkali Kurti</t>
-  </si>
-  <si>
-    <t>DROPPED</t>
   </si>
   <si>
     <t>https://www.amazon.in/dp/B0H1R6YTDV</t>
@@ -82,13 +79,55 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="8">
     <font>
       <sz val="11.0"/>
       <color indexed="8"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="11.0"/>
+      <u val="single"/>
+      <color indexed="12"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="11.0"/>
+      <u val="single"/>
+      <color indexed="12"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="11.0"/>
+      <u val="single"/>
+      <color indexed="12"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="11.0"/>
+      <u val="single"/>
+      <color indexed="12"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="11.0"/>
+      <u val="single"/>
+      <color indexed="12"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="11.0"/>
+      <u val="single"/>
+      <color indexed="12"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="11.0"/>
+      <u val="single"/>
+      <color indexed="12"/>
     </font>
   </fonts>
   <fills count="2">
@@ -111,22 +150,29 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="true"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="true"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="true"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true"/>
   </cellXfs>
 </styleSheet>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:E8"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
     <col min="1" max="1" width="17.39453125" customWidth="true" bestFit="true"/>
     <col min="2" max="2" width="10.51953125" customWidth="true" bestFit="true"/>
     <col min="3" max="3" width="11.49609375" customWidth="true" bestFit="true"/>
-    <col min="4" max="4" width="8.73828125" customWidth="true" bestFit="true"/>
-    <col min="5" max="5" width="34.9140625" customWidth="true" bestFit="true"/>
+    <col min="4" max="4" width="7.1640625" customWidth="true" bestFit="true"/>
+    <col min="5" max="5" width="34.984375" customWidth="true" bestFit="true"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -159,7 +205,7 @@
       <c r="D2" t="s" s="0">
         <v>6</v>
       </c>
-      <c r="E2" t="s" s="0">
+      <c r="E2" t="s" s="1">
         <v>7</v>
       </c>
     </row>
@@ -176,7 +222,7 @@
       <c r="D3" t="s" s="0">
         <v>6</v>
       </c>
-      <c r="E3" t="s" s="0">
+      <c r="E3" t="s" s="2">
         <v>9</v>
       </c>
     </row>
@@ -193,7 +239,7 @@
       <c r="D4" t="s" s="0">
         <v>6</v>
       </c>
-      <c r="E4" t="s" s="0">
+      <c r="E4" t="s" s="3">
         <v>11</v>
       </c>
     </row>
@@ -205,18 +251,18 @@
         <v>1000.0</v>
       </c>
       <c r="C5" t="n" s="0">
-        <v>798.0</v>
+        <v>1699.0</v>
       </c>
       <c r="D5" t="s" s="0">
+        <v>6</v>
+      </c>
+      <c r="E5" t="s" s="4">
         <v>13</v>
-      </c>
-      <c r="E5" t="s" s="0">
-        <v>14</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s" s="0">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B6" t="n" s="0">
         <v>100.0</v>
@@ -227,13 +273,13 @@
       <c r="D6" t="s" s="0">
         <v>6</v>
       </c>
-      <c r="E6" t="s" s="0">
-        <v>16</v>
+      <c r="E6" t="s" s="5">
+        <v>15</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s" s="0">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B7" t="n" s="0">
         <v>15000.0</v>
@@ -244,13 +290,13 @@
       <c r="D7" t="s" s="0">
         <v>6</v>
       </c>
-      <c r="E7" t="s" s="0">
-        <v>18</v>
+      <c r="E7" t="s" s="6">
+        <v>17</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s" s="0">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B8" t="n" s="0">
         <v>4000.0</v>
@@ -261,11 +307,20 @@
       <c r="D8" t="s" s="0">
         <v>6</v>
       </c>
-      <c r="E8" t="s" s="0">
-        <v>20</v>
+      <c r="E8" t="s" s="7">
+        <v>19</v>
       </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="E2" r:id="rId1"/>
+    <hyperlink ref="E3" r:id="rId2"/>
+    <hyperlink ref="E4" r:id="rId3"/>
+    <hyperlink ref="E5" r:id="rId4"/>
+    <hyperlink ref="E6" r:id="rId5"/>
+    <hyperlink ref="E7" r:id="rId6"/>
+    <hyperlink ref="E8" r:id="rId7"/>
+  </hyperlinks>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>
 </file>
</xml_diff>